<commit_message>
cuadros 1 11 70 103 ok
</commit_message>
<xml_diff>
--- a/output/resultado_personalizado.xlsx
+++ b/output/resultado_personalizado.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PN00105MM</t>
+          <t>PN00001MM</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -508,12 +508,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>PN00106MM</t>
+          <t>PN00002MM</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -525,12 +525,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PN00107MM</t>
+          <t>PN00003MM</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -542,12 +542,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PN00108MM</t>
+          <t>PN00004MM</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -559,357 +559,353 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PN00110MM</t>
+          <t>PN00005MM</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>II. ACTIVOS EXTERNOS NETOS DE LARGO PLAZO &gt; (Millones de USD) 2/</t>
+          <t>II. ACTIVOS EXTERNOS NETOS DE LARGO PLAZO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PN00111MM</t>
+          <t>PN00006MM</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4)</t>
+          <t>II. ACTIVOS EXTERNOS NETOS DE LARGO PLAZO &gt; (Millones de USD) 2/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PN00112MM</t>
+          <t>PN00007MM</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto)</t>
+          <t>III. ACTIVOS INTERNOS NETOS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>PN00113MM</t>
-        </is>
-      </c>
+          <t>cuadro-001</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 1. Sector público</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PN00114MM</t>
+          <t>PN00009MM</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central &gt; - Créditos</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 1. Sector público &gt; a. En moneda nacional</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PN00115MM</t>
+          <t>PN00010MM</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central &gt; - Obligaciones</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 1. Sector público &gt; b. En moneda extranjera</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PN00116MM</t>
+          <t>PN00011MM</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 1. Sector público &gt; b. En moneda extranjera &gt; (millones de USD)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PN00117MM</t>
+          <t>PN00012MM</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/ &gt; - Créditos</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 2. Crédito al Sector Privado</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PN00118MM</t>
+          <t>PN00013MM</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/ &gt; - Obligaciones</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 2. Crédito al Sector Privado &gt; a. En moneda nacional</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PN00119MM</t>
+          <t>PN00014MM</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 2. Sector Privado</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 2. Crédito al Sector Privado &gt; b. En moneda extranjera</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PN00120MM</t>
+          <t>PN00015MM</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 2. Crédito al Sector Privado &gt; b. En moneda extranjera &gt; (millones de USD)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PN00121MM</t>
+          <t>PN00016MM</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP</t>
+          <t>III. ACTIVOS INTERNOS NETOS &gt; 3. Otras Cuentas</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PN00122MM</t>
+          <t>PN00017MM</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PN00123MM</t>
+          <t>PN00018MM</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 1. Moneda Nacional</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PN00124MM</t>
+          <t>PN00019MM</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Nacional</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 1. Moneda Nacional &gt; a. Dinero 4/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>PN00125MM</t>
+          <t>PN00020MM</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores &gt; * Cuenta corriente</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 1. Moneda Nacional &gt; a. Dinero 4/ &gt; i. Circulante</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PN00126MM</t>
+          <t>PN00021MM</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores &gt; * Otros depósitos 4/</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 1. Moneda Nacional &gt; a. Dinero 4/ &gt; ii. Depósitos a la Vista</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PN00127MM</t>
+          <t>PN00022MM</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores &gt; - Valores del BCRP</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 1. Moneda Nacional &gt; b. Cuasidinero</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>PN00128MM</t>
+          <t>PN00023MM</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Extranjera</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 2. Moneda Extranjera</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>PN00129MM</t>
+          <t>PN00024MM</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Efectivo &gt; iii. Obligaciones</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 2. Moneda Extranjera &gt; (Millones de USD)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>cuadro-011</t>
+          <t>cuadro-001</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>PN00130MM</t>
+          <t>PN00025MM</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; b. Banco de la Nación</t>
+          <t>IV. LIQUIDEZ (=I+II+III) 3/ &gt; 2. Moneda Extranjera &gt; Coeficiente de dolarización</t>
         </is>
       </c>
     </row>
@@ -921,12 +917,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PN00131MM</t>
+          <t>PN00105MM</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Créditos y Depósitos</t>
+          <t>I. ACTIVOS EXTERNOS NETOS DE CORTO PLAZO</t>
         </is>
       </c>
     </row>
@@ -938,12 +934,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PN00132MM</t>
+          <t>PN00106MM</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; i. Créditos y Depósitos &gt; ii. Obligaciones</t>
+          <t>I. ACTIVOS EXTERNOS NETOS DE CORTO PLAZO &gt; (Millones de USD)</t>
         </is>
       </c>
     </row>
@@ -955,12 +951,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PN00134MM</t>
+          <t>PN00107MM</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 4. Otras Cuentas Netas</t>
+          <t>I. ACTIVOS EXTERNOS NETOS DE CORTO PLAZO &gt; 1. Activos</t>
         </is>
       </c>
     </row>
@@ -972,12 +968,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>PN00135MM</t>
+          <t>PN00108MM</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III)</t>
+          <t>I. ACTIVOS EXTERNOS NETOS DE CORTO PLAZO &gt; 2. Pasivos</t>
         </is>
       </c>
     </row>
@@ -989,12 +985,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>PN00136MM</t>
+          <t>PN00109MM</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional</t>
+          <t>II. ACTIVOS EXTERNOS NETOS DE LARGO PLAZO</t>
         </is>
       </c>
     </row>
@@ -1006,12 +1002,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>PN00137MM</t>
+          <t>PN00110MM</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; a. Obligaciones a la Vista</t>
+          <t>II. ACTIVOS EXTERNOS NETOS DE LARGO PLAZO &gt; (Millones de USD) 2/</t>
         </is>
       </c>
     </row>
@@ -1023,12 +1019,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>PN00138MM</t>
+          <t>PN00111MM</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; b. Obligaciones de Ahorro</t>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4)</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1036,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>PN00139MM</t>
+          <t>PN00112MM</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; c. Obligaciones a Plazo</t>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto)</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1053,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>PN00140MM</t>
+          <t>PN00113MM</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; d. Otros Valores</t>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central</t>
         </is>
       </c>
     </row>
@@ -1074,12 +1070,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>PN00141MM</t>
+          <t>PN00114MM</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera</t>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central &gt; - Créditos</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1087,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>PN00142MM</t>
+          <t>PN00115MM</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera &gt; (Millones de USD)</t>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; a. Gobierno Central &gt; - Obligaciones</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1104,2300 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>PN00116MM</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>PN00117MM</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/ &gt; - Créditos</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>PN00118MM</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 1. Sector Público (neto) &gt; b. Resto Sector Público 3/ &gt; - Obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>PN00119MM</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 2. Sector Privado</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>PN00120MM</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>PN00121MM</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>PN00122MM</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; i. Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>PN00123MM</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>PN00124MM</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>PN00125MM</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Nacional &gt; * Cuenta corriente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>PN00126MM</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Nacional &gt; * Otros depósitos 4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>PN00127MM</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores &gt; - Valores del BCRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>PN00128MM</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; ii. Depósitos y valores &gt; - Depósitos en Moneda Extranjera</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>PN00129MM</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; a. BCRP &gt; iii. Obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>PN00130MM</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; b. Banco de la Nación</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>PN00131MM</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; b. Banco de la Nación &gt; i. Créditos y Depósitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>PN00132MM</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 3. Operaciones Interbancarias &gt; b. Banco de la Nación &gt; ii. Obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>PN00134MM</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>III. ACTIVOS INTERNOS NETOS (1+2+3+4) &gt; 4. Otras Cuentas Netas</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>PN00135MM</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>PN00136MM</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>PN00137MM</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; a. Obligaciones a la Vista</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>PN00138MM</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; b. Obligaciones de Ahorro</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>PN00139MM</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; c. Obligaciones a Plazo</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>PN00140MM</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 1 En Moneda Nacional &gt; d. Otros Valores</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>PN00141MM</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>PN00142MM</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera &gt; (Millones de USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-011</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
           <t>PN00143MM</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera &gt; Coeficiente de dolarización de la liquidez (%)</t>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>IV. LIQUIDEZ (I+II+III) &gt; 2. En Moneda Extranjera &gt; Coeficiente de dolarización</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Productos primarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Arándanos</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Uvas</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Café</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Paltas</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Cacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Espárragos</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Mangos</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Mandarinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n"/>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Manufacturas de origen agrícola</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Conservas de frutas y hortalizas</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Manufacturas de cacao y confitería</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Frutas congeladas</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Aceites y grasas vegetales y animales</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Alimento para animales</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Panadería y molinería</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Harina de pescado</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Pota</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Aceite de pescado</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Langostinos</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Extracción de minerales metálicos, no metálicos y carbón</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Cobre concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Plomo concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Zinc concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Oro concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Molibdeno concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Hierro, lodos y tortas</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n"/>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Fosfatos de calcio</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n"/>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Carbón</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n"/>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n"/>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Manufacturas de metales, minerales no metálicos y hierro</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n"/>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Oro doré</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n"/>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Cobre refinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n"/>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Estaño</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="n"/>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de cobre</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="n"/>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Zinc refinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="n"/>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de zinc</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="n"/>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de plata</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="n"/>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de hierro</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="n"/>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="n"/>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="n"/>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Derivados de petróleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="n"/>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="n"/>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Petróleo crudo</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="n"/>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="n"/>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Prendas de vestir, fibras y productos textiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="n"/>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; T-shirts de algodón</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="n"/>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Camisas de algodón para hombres</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="n"/>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Pelo fino de auquénidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="n"/>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="n"/>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Fabricación de sustancias y productos químicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="n"/>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Tintas y colorantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="n"/>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Ácido sulfúrico</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="n"/>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Etanol</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="n"/>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="n"/>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Fabricación de productos de plástico y caucho</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="n"/>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Películas de propileno</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="n"/>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Películas de etileno</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="n"/>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="n"/>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Productos elaborados de metal, excepto maquinaria y equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="n"/>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Maquinaria y equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="n"/>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Joyas y bisutería</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="n"/>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="n"/>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>6. Otras exportaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-070</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="n"/>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>6. Otras exportaciones &gt; TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="n"/>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="n"/>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Productos primarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="n"/>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Arándanos</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="n"/>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Uvas</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="n"/>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Café</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="n"/>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Paltas</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="n"/>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Cacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="n"/>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Espárragos</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="n"/>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Mangos</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="n"/>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Mandarinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="n"/>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="n"/>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Manufacturas de origen agrícola</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="n"/>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Conservas de frutas y hortalizas</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="n"/>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Manufacturas de cacao y confitería</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="n"/>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Frutas congeladas</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="n"/>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Aceites y grasas vegetales y animales</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="n"/>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Alimento para animales</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="n"/>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Panadería y molinería</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="n"/>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>1. Agropecuario &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="n"/>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="n"/>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Harina de pescado</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="n"/>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Pota</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="n"/>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Aceite de pescado</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="n"/>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Langostinos</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="n"/>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>2. Pesca y sus manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="n"/>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="n"/>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Extracción de minerales metálicos, no metálicos y carbón</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="n"/>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Cobre concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="n"/>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Plomo concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="n"/>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Zinc concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="n"/>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Oro concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="n"/>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Molibdeno concentrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="n"/>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Hierro, lodos y tortas</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="n"/>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Fosfatos de calcio</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="n"/>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Carbón</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="n"/>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="n"/>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Manufacturas de metales, minerales no metálicos y hierro</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="n"/>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Oro doré</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="n"/>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Cobre refinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="n"/>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Estaño</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="n"/>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de cobre</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="n"/>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Zinc refinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="n"/>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de zinc</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="n"/>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de plata</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="n"/>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Productos de hierro</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="n"/>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>3. Minería metálica y no metálica y sus manufacturas 2/ 3/ &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="n"/>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="n"/>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Derivados de petróleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="n"/>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="n"/>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>4. Extracción y refinación de petróleo y gas natural &gt; Petróleo crudo</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="n"/>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="n"/>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Prendas de vestir, fibras y productos textiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="n"/>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; T-shirts de algodón</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="n"/>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Camisas de algodón para hombres</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="n"/>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Pelo fino de auquénidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="n"/>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="n"/>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Fabricación de sustancias y productos químicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="n"/>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Tintas y colorantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="n"/>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Ácido sulfúrico</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="n"/>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Etanol</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="n"/>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="n"/>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Fabricación de productos de plástico y caucho</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="n"/>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Películas de propileno</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="n"/>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Películas de etileno</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="n"/>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="n"/>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Productos elaborados de metal, excepto maquinaria y equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="n"/>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Maquinaria y equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="n"/>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Joyas y bisutería</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="n"/>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>5. Resto de manufacturas &gt; Resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="n"/>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>6. Otras exportaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>cuadro-103</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="n"/>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>6. Otras exportaciones &gt; TOTAL</t>
         </is>
       </c>
     </row>

</xml_diff>